<commit_message>
Move lookup lesson and simplify raw data example
</commit_message>
<xml_diff>
--- a/textbook_examples/elevator_tickets_correct.xlsx
+++ b/textbook_examples/elevator_tickets_correct.xlsx
@@ -1,8 +1,8 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10817"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30413"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pjs998/Downloads/"/>
@@ -19,7 +19,7 @@
   <definedNames>
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">elevator_tickets!$A$1:$G$21</definedName>
   </definedNames>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -279,7 +279,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -308,9 +308,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -324,7 +323,7 @@
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="19" formatCode="yyyy/mm/dd"/>
+      <numFmt numFmtId="164" formatCode="yyyy/mm/dd"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
@@ -698,17 +697,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{98AA78CB-85E8-2345-9AF0-D11C9C5B3B7A}">
   <dimension ref="A1:G21"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <cols>
-    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="14.5" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.83203125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.6640625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -731,463 +730,463 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:7">
+      <c r="A2" t="s">
         <v>7</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" t="s">
         <v>8</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" t="s">
         <v>9</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="1">
         <v>45957</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" t="s">
         <v>10</v>
       </c>
       <c r="F2">
         <v>24.3</v>
       </c>
-      <c r="G2" s="1" t="s">
+      <c r="G2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:7">
+      <c r="A3" t="s">
         <v>12</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" t="s">
         <v>13</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="C3" t="s">
         <v>14</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="1">
         <v>45914</v>
       </c>
-      <c r="E3" s="1" t="s">
+      <c r="E3" t="s">
         <v>15</v>
       </c>
       <c r="F3">
         <v>24</v>
       </c>
-      <c r="G3" s="1" t="s">
+      <c r="G3" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:7">
+      <c r="A4" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" s="1" t="s">
+      <c r="C4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="1">
         <v>45892</v>
       </c>
-      <c r="E4" s="1" t="s">
+      <c r="E4" t="s">
         <v>20</v>
       </c>
       <c r="F4">
         <v>28.4</v>
       </c>
-      <c r="G4" s="1" t="s">
+      <c r="G4" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:7">
+      <c r="A5" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="1" t="s">
+      <c r="C5" t="s">
         <v>23</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="1">
         <v>45945</v>
       </c>
-      <c r="E5" s="1" t="s">
+      <c r="E5" t="s">
         <v>20</v>
       </c>
       <c r="F5">
         <v>18.899999999999999</v>
       </c>
-      <c r="G5" s="1" t="s">
+      <c r="G5" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:7">
+      <c r="A6" t="s">
         <v>24</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="1" t="s">
+      <c r="C6" t="s">
         <v>26</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="1">
         <v>45936</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="E6" t="s">
         <v>27</v>
       </c>
       <c r="F6">
         <v>21.6</v>
       </c>
-      <c r="G6" s="1" t="s">
+      <c r="G6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:7">
+      <c r="A7" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="1" t="s">
+      <c r="C7" t="s">
         <v>30</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="1">
         <v>45920</v>
       </c>
-      <c r="E7" s="1" t="s">
+      <c r="E7" t="s">
         <v>15</v>
       </c>
       <c r="F7">
         <v>30.2</v>
       </c>
-      <c r="G7" s="1" t="s">
+      <c r="G7" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:7">
+      <c r="A8" t="s">
         <v>32</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="1" t="s">
+      <c r="C8" t="s">
         <v>34</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="1">
         <v>45880</v>
       </c>
-      <c r="E8" s="1" t="s">
+      <c r="E8" t="s">
         <v>10</v>
       </c>
       <c r="F8">
         <v>38.9</v>
       </c>
-      <c r="G8" s="1" t="s">
+      <c r="G8" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:7">
+      <c r="A9" t="s">
         <v>35</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" t="s">
         <v>36</v>
       </c>
-      <c r="C9" s="1" t="s">
+      <c r="C9" t="s">
         <v>37</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="1">
         <v>45932</v>
       </c>
-      <c r="E9" s="1" t="s">
+      <c r="E9" t="s">
         <v>15</v>
       </c>
       <c r="F9">
         <v>37.799999999999997</v>
       </c>
-      <c r="G9" s="1" t="s">
+      <c r="G9" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:7">
+      <c r="A10" t="s">
         <v>38</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" t="s">
         <v>39</v>
       </c>
-      <c r="C10" s="1" t="s">
+      <c r="C10" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="1">
         <v>45949</v>
       </c>
-      <c r="E10" s="1" t="s">
+      <c r="E10" t="s">
         <v>20</v>
       </c>
       <c r="F10">
         <v>28.3</v>
       </c>
-      <c r="G10" s="1" t="s">
+      <c r="G10" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:7">
+      <c r="A11" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="C11" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="1">
         <v>45897</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="E11" t="s">
         <v>15</v>
       </c>
       <c r="F11">
         <v>23.2</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="G11" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:7">
+      <c r="A12" t="s">
         <v>44</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" t="s">
         <v>45</v>
       </c>
-      <c r="C12" s="1" t="s">
+      <c r="C12" t="s">
         <v>46</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="1">
         <v>45896</v>
       </c>
-      <c r="E12" s="1" t="s">
+      <c r="E12" t="s">
         <v>20</v>
       </c>
       <c r="F12">
         <v>31.8</v>
       </c>
-      <c r="G12" s="1" t="s">
+      <c r="G12" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:7">
+      <c r="A13" t="s">
         <v>47</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" t="s">
         <v>48</v>
       </c>
-      <c r="C13" s="1" t="s">
+      <c r="C13" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="1">
         <v>45925</v>
       </c>
-      <c r="E13" s="1" t="s">
+      <c r="E13" t="s">
         <v>27</v>
       </c>
       <c r="F13">
         <v>31.5</v>
       </c>
-      <c r="G13" s="1" t="s">
+      <c r="G13" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:7">
+      <c r="A14" t="s">
         <v>49</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" t="s">
         <v>50</v>
       </c>
-      <c r="C14" s="1" t="s">
+      <c r="C14" t="s">
         <v>51</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="1">
         <v>45889</v>
       </c>
-      <c r="E14" s="1" t="s">
+      <c r="E14" t="s">
         <v>10</v>
       </c>
       <c r="F14">
         <v>19.5</v>
       </c>
-      <c r="G14" s="1" t="s">
+      <c r="G14" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:7">
+      <c r="A15" t="s">
         <v>52</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" t="s">
         <v>53</v>
       </c>
-      <c r="C15" s="1" t="s">
+      <c r="C15" t="s">
         <v>54</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="1">
         <v>45884</v>
       </c>
-      <c r="E15" s="1" t="s">
+      <c r="E15" t="s">
         <v>15</v>
       </c>
       <c r="F15">
         <v>33.799999999999997</v>
       </c>
-      <c r="G15" s="1" t="s">
+      <c r="G15" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="1" t="s">
+    <row r="16" spans="1:7">
+      <c r="A16" t="s">
         <v>55</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" t="s">
         <v>56</v>
       </c>
-      <c r="C16" s="1" t="s">
+      <c r="C16" t="s">
         <v>57</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="1">
         <v>45890</v>
       </c>
-      <c r="E16" s="1" t="s">
+      <c r="E16" t="s">
         <v>27</v>
       </c>
       <c r="F16">
         <v>30.5</v>
       </c>
-      <c r="G16" s="1" t="s">
+      <c r="G16" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A17" s="1" t="s">
+    <row r="17" spans="1:7">
+      <c r="A17" t="s">
         <v>58</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" t="s">
         <v>59</v>
       </c>
-      <c r="C17" s="1" t="s">
+      <c r="C17" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="1">
         <v>45953</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="E17" t="s">
         <v>27</v>
       </c>
       <c r="F17">
         <v>40.5</v>
       </c>
-      <c r="G17" s="1" t="s">
+      <c r="G17" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A18" s="1" t="s">
+    <row r="18" spans="1:7">
+      <c r="A18" t="s">
         <v>61</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" t="s">
         <v>62</v>
       </c>
-      <c r="C18" s="1" t="s">
+      <c r="C18" t="s">
         <v>63</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="1">
         <v>45884</v>
       </c>
-      <c r="E18" s="1" t="s">
+      <c r="E18" t="s">
         <v>10</v>
       </c>
       <c r="F18">
         <v>36.1</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
+    <row r="19" spans="1:7">
+      <c r="A19" t="s">
         <v>64</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" t="s">
         <v>65</v>
       </c>
-      <c r="C19" s="1" t="s">
+      <c r="C19" t="s">
         <v>66</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="1">
         <v>45953</v>
       </c>
-      <c r="E19" s="1" t="s">
+      <c r="E19" t="s">
         <v>27</v>
       </c>
       <c r="F19">
         <v>29</v>
       </c>
-      <c r="G19" s="1" t="s">
+      <c r="G19" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A20" s="1" t="s">
+    <row r="20" spans="1:7">
+      <c r="A20" t="s">
         <v>67</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" t="s">
         <v>68</v>
       </c>
-      <c r="C20" s="1" t="s">
+      <c r="C20" t="s">
         <v>69</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="1">
         <v>45937</v>
       </c>
-      <c r="E20" s="1" t="s">
+      <c r="E20" t="s">
         <v>70</v>
       </c>
       <c r="F20">
         <v>25.9</v>
       </c>
-      <c r="G20" s="1" t="s">
+      <c r="G20" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A21" s="1" t="s">
+    <row r="21" spans="1:7">
+      <c r="A21" t="s">
         <v>71</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" t="s">
         <v>72</v>
       </c>
-      <c r="C21" s="1" t="s">
+      <c r="C21" t="s">
         <v>73</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="1">
         <v>45906</v>
       </c>
-      <c r="E21" s="1" t="s">
+      <c r="E21" t="s">
         <v>70</v>
       </c>
       <c r="F21">
         <v>25.1</v>
       </c>
-      <c r="G21" s="1" t="s">
+      <c r="G21" t="s">
         <v>31</v>
       </c>
     </row>
@@ -1202,7 +1201,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5E67A241-BD77-E246-A06B-549FF49391CA}">
   <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.95"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1212,9 +1211,5 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9440673-5CF1-1F46-93F7-37F0BE526FB9}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/DataMashup"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D9440673-5CF1-1F46-93F7-37F0BE526FB9}"/>
 </file>
</xml_diff>